<commit_message>
District Report (Excel): add the District Report table as the first sheet
The "District Report (Excel)" download now opens on a "District Report"
sheet in the layout from the district report review: one row per block
with schools and students assessed, overall, Grade 5 and Grade 8 scores,
subject scores (Odia, English, Maths for both grades; EVS for Grade 5;
Science and Social Science for Grade 8), schools with recoverable points,
schools above their block's average, the three weakest and three best
learning outcomes, and schools by band. Scores carry a red-yellow-green
heat map per column, with a district total row and a short legend.

The Blocks, Schools and Subjects by block sheets follow unchanged. Rows
come from block_report.csv, so run build_district_competencies.py before
build_district_report.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01H1sRStbh28mbP4JKTzFN2R
</commit_message>
<xml_diff>
--- a/public/data/downloads/district_report.xlsx
+++ b/public/data/downloads/district_report.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocks" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schools" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subjects by block" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="District Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Blocks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Schools" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Subjects by block" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,8 +19,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0&quot;%&quot;"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,17 +32,59 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="002D3A47"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00566579"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002D3A47"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C24E36"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B5530C"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00A85A0F"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0015803D"/>
+    </font>
+    <font>
+      <color rgb="00566579"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E9ECEE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3EFE8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,13 +92,82 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9CED3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C9CED3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9CED3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9CED3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,6 +533,1150 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:X19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
+    <col width="30" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Anugola District: SAKSHAM District Report</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Grade 5 and Grade 8, 2025-26. Scores are the share of answers correct (%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>S. No.</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Block Name</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Schools Assessed</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Students Assessed</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Overall Score</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Grade 5 Score</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Grade 8 Score</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Odia</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Maths</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>EVS (only G5)</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Science (only G8)</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Social Science (only G8)</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>No. of schools with recoverable points</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>No. of schools scoring above their block's average</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>Weakest learning outcomes in this block (top 3)</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Best performing learning outcomes in this block (top 3)</t>
+        </is>
+      </c>
+      <c r="U3" s="3" t="inlineStr">
+        <is>
+          <t>Number of schools by band</t>
+        </is>
+      </c>
+      <c r="V3" s="3" t="n"/>
+      <c r="W3" s="3" t="n"/>
+      <c r="X3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n"/>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>Needs Support</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>Developing</t>
+        </is>
+      </c>
+      <c r="X4" s="3" t="inlineStr">
+        <is>
+          <t>Excelling</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Anugola</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>188</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>4761</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>59.8</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>49.5</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>65.5</v>
+      </c>
+      <c r="N5" s="6" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>50.1</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>60.3</v>
+      </c>
+      <c r="Q5" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="R5" s="4" t="n">
+        <v>122</v>
+      </c>
+      <c r="S5" s="7" t="inlineStr">
+        <is>
+          <t>SCI 716 (35%); OD 716 (37%); SST 717 (37%)</t>
+        </is>
+      </c>
+      <c r="T5" s="7" t="inlineStr">
+        <is>
+          <t>OD 806 (89%); M 803 (85%); OD 407 (84%)</t>
+        </is>
+      </c>
+      <c r="U5" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" s="9" t="n">
+        <v>20</v>
+      </c>
+      <c r="W5" s="10" t="n">
+        <v>119</v>
+      </c>
+      <c r="X5" s="11" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Athamallik</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>194</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>3437</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>62.1</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>71.09999999999999</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>58.9</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>64.09999999999999</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>59.4</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>67.09999999999999</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="N6" s="6" t="n">
+        <v>60.8</v>
+      </c>
+      <c r="O6" s="6" t="n">
+        <v>58.4</v>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="Q6" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="R6" s="4" t="n">
+        <v>110</v>
+      </c>
+      <c r="S6" s="7" t="inlineStr">
+        <is>
+          <t>SST 717 (37%); E 501 (44%); M 721 (44%)</t>
+        </is>
+      </c>
+      <c r="T6" s="7" t="inlineStr">
+        <is>
+          <t>E 408 (85%); E 405 (85%); OD 507 (83%)</t>
+        </is>
+      </c>
+      <c r="U6" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V6" s="9" t="n">
+        <v>29</v>
+      </c>
+      <c r="W6" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="X6" s="11" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Banarpal</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>3848</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>57.2</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>49.8</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>52.3</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>69.7</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="N7" s="6" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>51.6</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="Q7" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="R7" s="4" t="n">
+        <v>104</v>
+      </c>
+      <c r="S7" s="7" t="inlineStr">
+        <is>
+          <t>M 721 (22%); M 714 (28%); M 711 (29%)</t>
+        </is>
+      </c>
+      <c r="T7" s="7" t="inlineStr">
+        <is>
+          <t>OD 806 (88%); M 419 (86%); M 420 (85%)</t>
+        </is>
+      </c>
+      <c r="U7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>31</v>
+      </c>
+      <c r="W7" s="10" t="n">
+        <v>97</v>
+      </c>
+      <c r="X7" s="11" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Chhendipada</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="n">
+        <v>178</v>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>4036</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>62.8</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>66.59999999999999</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>59.5</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="N8" s="6" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>60.9</v>
+      </c>
+      <c r="Q8" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="R8" s="4" t="n">
+        <v>108</v>
+      </c>
+      <c r="S8" s="7" t="inlineStr">
+        <is>
+          <t>SST 832 (39%); EN 710 (41%); M 721 (45%)</t>
+        </is>
+      </c>
+      <c r="T8" s="7" t="inlineStr">
+        <is>
+          <t>OD 806 (89%); SST 708 (88%); M 811 (86%)</t>
+        </is>
+      </c>
+      <c r="U8" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V8" s="9" t="n">
+        <v>23</v>
+      </c>
+      <c r="W8" s="10" t="n">
+        <v>110</v>
+      </c>
+      <c r="X8" s="11" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Kaniha</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>153</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>2976</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>71</v>
+      </c>
+      <c r="N9" s="6" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>68.59999999999999</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="Q9" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="R9" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="S9" s="7" t="inlineStr">
+        <is>
+          <t>SST 717 (36%); OD 716 (38%); SST 832 (38%)</t>
+        </is>
+      </c>
+      <c r="T9" s="7" t="inlineStr">
+        <is>
+          <t>M 803 (90%); E 405 (90%); SST 825 (88%)</t>
+        </is>
+      </c>
+      <c r="U9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V9" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="W9" s="10" t="n">
+        <v>92</v>
+      </c>
+      <c r="X9" s="11" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Kishorenagar</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>157</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>3024</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>65.8</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>72.09999999999999</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>56.3</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>68.90000000000001</v>
+      </c>
+      <c r="N10" s="6" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="O10" s="6" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>97</v>
+      </c>
+      <c r="S10" s="7" t="inlineStr">
+        <is>
+          <t>M 721 (39%); SST 717 (41%); E 415 (45%)</t>
+        </is>
+      </c>
+      <c r="T10" s="7" t="inlineStr">
+        <is>
+          <t>OD 806 (88%); M 803 (88%); M 420 (88%)</t>
+        </is>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="V10" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="W10" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="X10" s="11" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Palalahada</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>3799</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>65.59999999999999</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>59.3</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>69</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>59.1</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>68.3</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="N11" s="6" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>105</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>115</v>
+      </c>
+      <c r="S11" s="7" t="inlineStr">
+        <is>
+          <t>M 721 (31%); SST 717 (31%); SST 832 (40%)</t>
+        </is>
+      </c>
+      <c r="T11" s="7" t="inlineStr">
+        <is>
+          <t>OD 806 (87%); SST 708 (85%); M 803 (83%)</t>
+        </is>
+      </c>
+      <c r="U11" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" s="9" t="n">
+        <v>41</v>
+      </c>
+      <c r="W11" s="10" t="n">
+        <v>136</v>
+      </c>
+      <c r="X11" s="11" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Talacher</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="n">
+        <v>112</v>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2198</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>64.40000000000001</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>56.9</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>54.7</v>
+      </c>
+      <c r="N12" s="6" t="n">
+        <v>57.4</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="P12" s="6" t="n">
+        <v>53.3</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="S12" s="7" t="inlineStr">
+        <is>
+          <t>M 721 (30%); SCI 709 (32%); SCI 712 (33%)</t>
+        </is>
+      </c>
+      <c r="T12" s="7" t="inlineStr">
+        <is>
+          <t>SST 708 (85%); OD 806 (83%); OD 407 (78%)</t>
+        </is>
+      </c>
+      <c r="U12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="V12" s="9" t="n">
+        <v>28</v>
+      </c>
+      <c r="W12" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="X12" s="11" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="12" t="inlineStr"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Total (district)</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="n">
+        <v>1361</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>28079</v>
+      </c>
+      <c r="E13" s="14" t="n">
+        <v>62</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>66.8</v>
+      </c>
+      <c r="G13" s="14" t="n">
+        <v>58.3</v>
+      </c>
+      <c r="H13" s="14" t="n">
+        <v>70.8</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>60.5</v>
+      </c>
+      <c r="J13" s="14" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>55.1</v>
+      </c>
+      <c r="L13" s="14" t="n">
+        <v>68.7</v>
+      </c>
+      <c r="M13" s="14" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="N13" s="14" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="O13" s="14" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="P13" s="14" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="Q13" s="12" t="n">
+        <v>538</v>
+      </c>
+      <c r="R13" s="12" t="n">
+        <v>817</v>
+      </c>
+      <c r="S13" s="15" t="inlineStr">
+        <is>
+          <t>M 721 (38%); SST 717 (39%); OD 716 (40%)</t>
+        </is>
+      </c>
+      <c r="T13" s="15" t="inlineStr">
+        <is>
+          <t>OD 806 (87%); OD 407 (84%); M 419 (83%)</t>
+        </is>
+      </c>
+      <c r="U13" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="V13" s="17" t="n">
+        <v>182</v>
+      </c>
+      <c r="W13" s="18" t="n">
+        <v>840</v>
+      </c>
+      <c r="X13" s="19" t="n">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>How to read this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>Heat map: in each score column, red marks the lowest-scoring blocks, yellow the middle and green the highest. Colours compare the eight blocks with each other; the number is shown in every cell.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>Recoverable points: schools scoring below their block's average. Lifting these schools towards the average recovers the most points for the block and district score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>Bands (school overall score): Critical 0 to 25%, Needs Support 26 to 50%, Developing 51 to 75%, Excelling 76 to 100%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>Learning outcomes: code with the share of students answering correctly in brackets. Full descriptions are in learning_outcomes_by_block.csv.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="L3:M3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="S3:S4"/>
+    <mergeCell ref="T3:T4"/>
+    <mergeCell ref="U3:X3"/>
+    <mergeCell ref="H3:I3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="E5:E12">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F12">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:G12">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H5:H12">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I5:I12">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J12">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K5:K12">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:L12">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M5:M12">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N5:N12">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O12">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P5:P12">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -433,42 +1691,42 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>block</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>overall</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>g5</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>g8</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>schools</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>students</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>pct_below50</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="22" t="inlineStr">
         <is>
           <t>pct_proficient</t>
         </is>
@@ -815,7 +2073,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -834,37 +2092,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>udise</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>school_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>block</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>cluster</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>setting</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>score_out_of_10</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>students_assessed</t>
         </is>
@@ -51232,7 +52490,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51248,22 +52506,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>block</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>grade</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>pct_correct</t>
         </is>

</xml_diff>